<commit_message>
Rows with changes height shouldn't indicate that they also have a custom row style when the style is not specified. In case of a row with same style as worksheet but custom height, the missing row style is not displayed as a a worksheet style.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Misc/AdjustToContents.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Misc/AdjustToContents.xlsx
@@ -3401,12 +3401,12 @@
     <x:col min="2" max="2" width="28.190625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:2" customFormat="1" ht="41.5039" customHeight="1">
+    <x:row r="1" spans="1:2" ht="41.5039" customHeight="1">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:2" customFormat="1" ht="27.669267" customHeight="1">
+    <x:row r="2" spans="1:2" ht="27.669267" customHeight="1">
       <x:c r="A2" s="2" t="s">
         <x:v>1</x:v>
       </x:c>
@@ -3650,97 +3650,97 @@
   <x:dimension ref="A1:A19"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:1" customFormat="1" ht="304.361925" customHeight="1">
+    <x:row r="1" spans="1:1" ht="304.361925" customHeight="1">
       <x:c r="A1" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:1" customFormat="1" ht="15.218096" customHeight="1">
+    <x:row r="2" spans="1:1" ht="15.218096" customHeight="1">
       <x:c r="A2" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:1" customFormat="1" ht="7.609048" customHeight="1">
+    <x:row r="3" spans="1:1" ht="7.609048" customHeight="1">
       <x:c r="A3" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:1" customFormat="1" ht="16.063546" customHeight="1">
+    <x:row r="4" spans="1:1" ht="16.063546" customHeight="1">
       <x:c r="A4" s="5" t="s">
         <x:v>9</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:1" customFormat="1" ht="24.095319" customHeight="1">
+    <x:row r="5" spans="1:1" ht="24.095319" customHeight="1">
       <x:c r="A5" s="6" t="s">
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" spans="1:1" customFormat="1" ht="32.127092" customHeight="1">
+    <x:row r="6" spans="1:1" ht="32.127092" customHeight="1">
       <x:c r="A6" s="7" t="s">
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" spans="1:1" customFormat="1" ht="40.158865" customHeight="1">
+    <x:row r="7" spans="1:1" ht="40.158865" customHeight="1">
       <x:c r="A7" s="8" t="s">
         <x:v>12</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" spans="1:1" customFormat="1" ht="48.190638" customHeight="1">
+    <x:row r="8" spans="1:1" ht="48.190638" customHeight="1">
       <x:c r="A8" s="9" t="s">
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" spans="1:1" customFormat="1" ht="56.222411" customHeight="1">
+    <x:row r="9" spans="1:1" ht="56.222411" customHeight="1">
       <x:c r="A9" s="10" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" spans="1:1" customFormat="1" ht="64.254184" customHeight="1">
+    <x:row r="10" spans="1:1" ht="64.254184" customHeight="1">
       <x:c r="A10" s="11" t="s">
         <x:v>15</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" spans="1:1" customFormat="1" ht="72.285957" customHeight="1">
+    <x:row r="11" spans="1:1" ht="72.285957" customHeight="1">
       <x:c r="A11" s="12" t="s">
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" spans="1:1" customFormat="1" ht="80.31773" customHeight="1">
+    <x:row r="12" spans="1:1" ht="80.31773" customHeight="1">
       <x:c r="A12" s="13" t="s">
         <x:v>17</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" spans="1:1" customFormat="1" ht="88.349503" customHeight="1">
+    <x:row r="13" spans="1:1" ht="88.349503" customHeight="1">
       <x:c r="A13" s="14" t="s">
         <x:v>18</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" spans="1:1" customFormat="1" ht="96.381276" customHeight="1">
+    <x:row r="14" spans="1:1" ht="96.381276" customHeight="1">
       <x:c r="A14" s="15" t="s">
         <x:v>19</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" spans="1:1" customFormat="1" ht="104.413049" customHeight="1">
+    <x:row r="15" spans="1:1" ht="104.413049" customHeight="1">
       <x:c r="A15" s="16" t="s">
         <x:v>20</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" spans="1:1" customFormat="1" ht="112.444822" customHeight="1">
+    <x:row r="16" spans="1:1" ht="112.444822" customHeight="1">
       <x:c r="A16" s="17" t="s">
         <x:v>21</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" spans="1:1" customFormat="1" ht="120.476595" customHeight="1">
+    <x:row r="17" spans="1:1" ht="120.476595" customHeight="1">
       <x:c r="A17" s="18" t="s">
         <x:v>22</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" spans="1:1" customFormat="1" ht="128.508368" customHeight="1">
+    <x:row r="18" spans="1:1" ht="128.508368" customHeight="1">
       <x:c r="A18" s="19" t="s">
         <x:v>23</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" spans="1:1" customFormat="1" ht="136.540141" customHeight="1">
+    <x:row r="19" spans="1:1" ht="136.540141" customHeight="1">
       <x:c r="A19" s="20" t="s">
         <x:v>24</x:v>
       </x:c>
@@ -3762,97 +3762,97 @@
   <x:dimension ref="A1:A19"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:1" customFormat="1" ht="304.361925" customHeight="1">
+    <x:row r="1" spans="1:1" ht="304.361925" customHeight="1">
       <x:c r="A1" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:1" customFormat="1" ht="83.0078" customHeight="1">
+    <x:row r="2" spans="1:1" ht="83.0078" customHeight="1">
       <x:c r="A2" s="0" t="s">
         <x:v>43</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:1" customFormat="1" ht="17.293292" customHeight="1">
+    <x:row r="3" spans="1:1" ht="17.293292" customHeight="1">
       <x:c r="A3" s="4" t="s">
         <x:v>44</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:1" customFormat="1" ht="34.586583" customHeight="1">
+    <x:row r="4" spans="1:1" ht="34.586583" customHeight="1">
       <x:c r="A4" s="5" t="s">
         <x:v>45</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:1" customFormat="1" ht="51.879875" customHeight="1">
+    <x:row r="5" spans="1:1" ht="51.879875" customHeight="1">
       <x:c r="A5" s="6" t="s">
         <x:v>46</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" spans="1:1" customFormat="1" ht="69.173166" customHeight="1">
+    <x:row r="6" spans="1:1" ht="69.173166" customHeight="1">
       <x:c r="A6" s="7" t="s">
         <x:v>47</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" spans="1:1" customFormat="1" ht="86.466458" customHeight="1">
+    <x:row r="7" spans="1:1" ht="86.466458" customHeight="1">
       <x:c r="A7" s="8" t="s">
         <x:v>48</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" spans="1:1" customFormat="1" ht="103.759749" customHeight="1">
+    <x:row r="8" spans="1:1" ht="103.759749" customHeight="1">
       <x:c r="A8" s="9" t="s">
         <x:v>49</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" spans="1:1" customFormat="1" ht="121.053041" customHeight="1">
+    <x:row r="9" spans="1:1" ht="121.053041" customHeight="1">
       <x:c r="A9" s="10" t="s">
         <x:v>50</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" spans="1:1" customFormat="1" ht="138.346333" customHeight="1">
+    <x:row r="10" spans="1:1" ht="138.346333" customHeight="1">
       <x:c r="A10" s="11" t="s">
         <x:v>51</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" spans="1:1" customFormat="1" ht="155.639624" customHeight="1">
+    <x:row r="11" spans="1:1" ht="155.639624" customHeight="1">
       <x:c r="A11" s="12" t="s">
         <x:v>52</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" spans="1:1" customFormat="1" ht="172.932916" customHeight="1">
+    <x:row r="12" spans="1:1" ht="172.932916" customHeight="1">
       <x:c r="A12" s="13" t="s">
         <x:v>53</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" spans="1:1" customFormat="1" ht="190.226207" customHeight="1">
+    <x:row r="13" spans="1:1" ht="190.226207" customHeight="1">
       <x:c r="A13" s="14" t="s">
         <x:v>54</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" spans="1:1" customFormat="1" ht="207.519499" customHeight="1">
+    <x:row r="14" spans="1:1" ht="207.519499" customHeight="1">
       <x:c r="A14" s="15" t="s">
         <x:v>55</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" spans="1:1" customFormat="1" ht="224.81279" customHeight="1">
+    <x:row r="15" spans="1:1" ht="224.81279" customHeight="1">
       <x:c r="A15" s="16" t="s">
         <x:v>56</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" spans="1:1" customFormat="1" ht="242.106082" customHeight="1">
+    <x:row r="16" spans="1:1" ht="242.106082" customHeight="1">
       <x:c r="A16" s="17" t="s">
         <x:v>57</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" spans="1:1" customFormat="1" ht="259.399374" customHeight="1">
+    <x:row r="17" spans="1:1" ht="259.399374" customHeight="1">
       <x:c r="A17" s="18" t="s">
         <x:v>58</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" spans="1:1" customFormat="1" ht="276.692665" customHeight="1">
+    <x:row r="18" spans="1:1" ht="276.692665" customHeight="1">
       <x:c r="A18" s="19" t="s">
         <x:v>59</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" spans="1:1" customFormat="1" ht="293.985957" customHeight="1">
+    <x:row r="19" spans="1:1" ht="293.985957" customHeight="1">
       <x:c r="A19" s="20" t="s">
         <x:v>60</x:v>
       </x:c>

</xml_diff>